<commit_message>
Refresh market data and disclosures through 2026-10-16
</commit_message>
<xml_diff>
--- a/anthropic/2026-10-11/Anthropic_IPO_Basic_Valuation.xlsx
+++ b/anthropic/2026-10-11/Anthropic_IPO_Basic_Valuation.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation" sheetId="1" r:id="R587c4db865c54ea1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="2" r:id="R4435dffdbcd4489a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="3" r:id="R1abdb312155d4fa1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation" sheetId="1" r:id="Rcd6d0f44ea1e40f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="2" r:id="R46aee4bb4e8d4d23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="3" r:id="R7984c7315c3a422b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="10">
+  <x:numFmts count="13">
     <x:numFmt numFmtId="200" formatCode="#,##0.0;(#,##0.0);&quot;-&quot;"/>
     <x:numFmt numFmtId="201" formatCode="dd-mmm-yyyy"/>
     <x:numFmt numFmtId="202" formatCode="$#,##0.0;($#,##0.0);&quot;-&quot;"/>
@@ -26,6 +26,9 @@
     <x:numFmt numFmtId="207" formatCode="$0.000"/>
     <x:numFmt numFmtId="208" formatCode="0&quot;E&quot;"/>
     <x:numFmt numFmtId="209" formatCode="$0.00;($0.00);&quot;-&quot;"/>
+    <x:numFmt numFmtId="210" formatCode="0.0"/>
+    <x:numFmt numFmtId="211" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="212" formatCode="0.0%"/>
   </x:numFmts>
   <x:fonts count="20">
     <x:font>
@@ -199,7 +202,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="123">
+  <x:cellXfs count="127">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -563,6 +566,18 @@
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="202" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -920,7 +935,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0c48586677df4755"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc1d740eac1294e9c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -950,7 +965,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R44b75ae41e664c8b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8762bb2124e5426d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1348,15 +1363,15 @@
       <x:c r="A10" s="3"/>
       <x:c r="B10" s="3"/>
       <x:c r="C10" s="3" t="str">
-        <x:v>Reported IPO equity benchmark</x:v>
+        <x:v>IPO investor discussion</x:v>
       </x:c>
       <x:c r="D10" s="55" t="n">
         <x:f>'Inputs'!D15</x:f>
-        <x:v>2000</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="E10" s="4"/>
       <x:c r="F10" s="26" t="str">
-        <x:v>Reference target. Final offer price is unavailable.</x:v>
+        <x:v>Investor discussion; no priced offering or company valuation guidance.</x:v>
       </x:c>
       <x:c r="G10" s="4"/>
       <x:c r="H10" s="4"/>
@@ -1375,7 +1390,7 @@
       </x:c>
       <x:c r="D11" s="73" t="n">
         <x:f>D25/D10-1</x:f>
-        <x:v>-0.025000000000000022</x:v>
+        <x:v>0.30000000000000004</x:v>
       </x:c>
       <x:c r="E11" s="4"/>
       <x:c r="F11" s="26" t="str">
@@ -1398,7 +1413,7 @@
       </x:c>
       <x:c r="D12" s="73" t="n">
         <x:f>IF(ISNUMBER(D58),D58/D10-1,"n.a.")</x:f>
-        <x:v>-0.6057302778002258</x:v>
+        <x:v>-0.47430703706696764</x:v>
       </x:c>
       <x:c r="E12" s="4"/>
       <x:c r="F12" s="26" t="str">
@@ -1421,11 +1436,11 @@
       </x:c>
       <x:c r="D13" s="73" t="n">
         <x:f>D9/D10-1</x:f>
-        <x:v>-0.05714285714285727</x:v>
+        <x:v>0.2571428571428571</x:v>
       </x:c>
       <x:c r="E13" s="4"/>
       <x:c r="F13" s="26" t="str">
-        <x:v>Comps sits below the benchmark; DCF sits far below both.</x:v>
+        <x:v>Heterogeneous peer references; excluded from Zhipu transaction multiples.</x:v>
       </x:c>
       <x:c r="G13" s="4"/>
       <x:c r="H13" s="4"/>
@@ -1444,7 +1459,7 @@
       </x:c>
       <x:c r="D14" s="74" t="n">
         <x:f>(D10-D24)/D21</x:f>
-        <x:v>10.256410256410257</x:v>
+        <x:v>7.6923076923076925</x:v>
       </x:c>
       <x:c r="E14" s="4"/>
       <x:c r="F14" s="26" t="str">
@@ -2393,7 +2408,7 @@
       </x:c>
       <x:c r="K42" s="94" t="n">
         <x:f>(1+'Inputs'!$D$11)^(-K41)</x:f>
-        <x:v>0.4523492153368933</x:v>
+        <x:v>0.4523492153368934</x:v>
       </x:c>
       <x:c r="L42" s="94" t="n">
         <x:f>(1+'Inputs'!$D$11)^(-L41)</x:f>
@@ -2441,7 +2456,7 @@
       </x:c>
       <x:c r="K43" s="70" t="n">
         <x:f>K40*K42</x:f>
-        <x:v>45.91016441129217</x:v>
+        <x:v>45.91016441129218</x:v>
       </x:c>
       <x:c r="L43" s="70" t="n">
         <x:f>L40*L42</x:f>
@@ -2796,7 +2811,7 @@
       </x:c>
       <x:c r="D60" s="61" t="n">
         <x:f>IF('Inputs'!D11&gt;'Inputs'!D13,(D10-D24-D56)/N42*('Inputs'!D11-'Inputs'!D13),"n.a.")</x:f>
-        <x:v>464.8075623130818</x:v>
+        <x:v>325.0443929375923</x:v>
       </x:c>
       <x:c r="E60" s="4"/>
       <x:c r="F60" s="26" t="str">
@@ -2819,7 +2834,7 @@
       </x:c>
       <x:c r="D61" s="91" t="n">
         <x:f>IF(ISNUMBER(D60),(D60-SUM(D50:D52))/D46/(1-'Inputs'!D14),"n.a.")</x:f>
-        <x:v>1.1083558835579803</x:v>
+        <x:v>0.7953634877048167</x:v>
       </x:c>
       <x:c r="E61" s="4"/>
       <x:c r="F61" s="26" t="str">
@@ -3498,7 +3513,7 @@
       </x:c>
       <x:c r="E91" s="97" t="n">
         <x:f>IF(ISNUMBER(D91),D91/$D$10-1,"n.a.")</x:f>
-        <x:v>-0.6057302778002258</x:v>
+        <x:v>-0.47430703706696764</x:v>
       </x:c>
       <x:c r="F91" s="4"/>
       <x:c r="G91" s="4"/>
@@ -3522,7 +3537,7 @@
       </x:c>
       <x:c r="E92" s="97" t="n">
         <x:f>IF(ISNUMBER(D92),D92/$D$10-1,"n.a.")</x:f>
-        <x:v>-0.6098383604021655</x:v>
+        <x:v>-0.4797844805362207</x:v>
       </x:c>
       <x:c r="F92" s="4"/>
       <x:c r="G92" s="4"/>
@@ -3546,7 +3561,7 @@
       </x:c>
       <x:c r="E93" s="97" t="n">
         <x:f>IF(ISNUMBER(D93),D93/$D$10-1,"n.a.")</x:f>
-        <x:v>-0.05714285714285727</x:v>
+        <x:v>0.2571428571428571</x:v>
       </x:c>
       <x:c r="F93" s="4"/>
       <x:c r="G93" s="4"/>
@@ -3570,7 +3585,7 @@
       </x:c>
       <x:c r="E94" s="97" t="n">
         <x:f>IF(ISNUMBER(D94),D94/$D$10-1,"n.a.")</x:f>
-        <x:v>0.33119999999999994</x:v>
+        <x:v>0.7749333333333335</x:v>
       </x:c>
       <x:c r="F94" s="4"/>
       <x:c r="G94" s="4"/>
@@ -3594,7 +3609,7 @@
       </x:c>
       <x:c r="E95" s="121" t="n">
         <x:f>IF(ISNUMBER(D95),D95/$D$10-1,"n.a.")</x:f>
-        <x:v>-0.05714285714285727</x:v>
+        <x:v>0.2571428571428571</x:v>
       </x:c>
       <x:c r="F95" s="4"/>
       <x:c r="G95" s="4"/>
@@ -3618,7 +3633,7 @@
       </x:c>
       <x:c r="E96" s="97" t="n">
         <x:f>IF(ISNUMBER(D96),D96/$D$10-1,"n.a.")</x:f>
-        <x:v>-0.5175000000000001</x:v>
+        <x:v>-0.3566666666666667</x:v>
       </x:c>
       <x:c r="F96" s="4"/>
       <x:c r="G96" s="4"/>
@@ -3642,7 +3657,7 @@
       </x:c>
       <x:c r="E97" s="97" t="n">
         <x:f>IF(ISNUMBER(D97),D97/$D$10-1,"n.a.")</x:f>
-        <x:v>-0.44999999999999996</x:v>
+        <x:v>-0.2666666666666667</x:v>
       </x:c>
       <x:c r="F97" s="4"/>
       <x:c r="G97" s="4"/>
@@ -3666,7 +3681,7 @@
       </x:c>
       <x:c r="E98" s="97" t="n">
         <x:f>IF(ISNUMBER(D98),D98/$D$10-1,"n.a.")</x:f>
-        <x:v>-0.09999999999999998</x:v>
+        <x:v>0.19999999999999996</x:v>
       </x:c>
       <x:c r="F98" s="4"/>
       <x:c r="G98" s="4"/>
@@ -3682,11 +3697,11 @@
       <x:c r="A99" s="3"/>
       <x:c r="B99" s="3"/>
       <x:c r="C99" s="3" t="str">
-        <x:v>IPO equity benchmark</x:v>
+        <x:v>IPO investor discussion</x:v>
       </x:c>
       <x:c r="D99" s="19" t="n">
         <x:f>D10</x:f>
-        <x:v>2000</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="E99" s="97" t="n">
         <x:f>IF(ISNUMBER(D99),D99/$D$10-1,"n.a.")</x:f>
@@ -3758,7 +3773,7 @@
       <x:c r="A103" s="3"/>
       <x:c r="B103" s="3"/>
       <x:c r="C103" s="9" t="str">
-        <x:v>The entire $2tn case rests on which peer tier the market assigns, not on the discount rate.</x:v>
+        <x:v>Latest investor discussion is USD1.5tn; the earlier USD2tn expectation is a historical stress case.</x:v>
       </x:c>
       <x:c r="D103" s="5"/>
       <x:c r="E103" s="5"/>
@@ -3841,7 +3856,9 @@
     <x:row r="108" ht="21" customHeight="1">
       <x:c r="A108" s="3"/>
       <x:c r="B108" s="3"/>
-      <x:c r="C108" s="3"/>
+      <x:c r="C108" s="3" t="str">
+        <x:v>Reported quarters and annual revenue assumption</x:v>
+      </x:c>
       <x:c r="D108" s="5"/>
       <x:c r="E108" s="5"/>
       <x:c r="F108" s="5"/>
@@ -3857,8 +3874,13 @@
     <x:row r="109" ht="21" customHeight="1">
       <x:c r="A109" s="3"/>
       <x:c r="B109" s="3"/>
-      <x:c r="C109" s="3"/>
-      <x:c r="D109" s="5"/>
+      <x:c r="C109" s="3" t="str">
+        <x:v>Reported Q1-Q3 revenue (USD bn)</x:v>
+      </x:c>
+      <x:c r="D109" s="125" t="n">
+        <x:f>SUM('Inputs'!J37:J39)</x:f>
+        <x:v>33.1</x:v>
+      </x:c>
       <x:c r="E109" s="5"/>
       <x:c r="F109" s="5"/>
       <x:c r="G109" s="5"/>
@@ -3873,8 +3895,13 @@
     <x:row r="110" ht="21" customHeight="1">
       <x:c r="A110" s="3"/>
       <x:c r="B110" s="3"/>
-      <x:c r="C110" s="3"/>
-      <x:c r="D110" s="5"/>
+      <x:c r="C110" s="3" t="str">
+        <x:v>FY2026 revenue assumption (USD bn)</x:v>
+      </x:c>
+      <x:c r="D110" s="125" t="n">
+        <x:f>'Inputs'!D22</x:f>
+        <x:v>64</x:v>
+      </x:c>
       <x:c r="E110" s="5"/>
       <x:c r="F110" s="5"/>
       <x:c r="G110" s="5"/>
@@ -3889,8 +3916,13 @@
     <x:row r="111" ht="21" customHeight="1">
       <x:c r="A111" s="3"/>
       <x:c r="B111" s="3"/>
-      <x:c r="C111" s="3"/>
-      <x:c r="D111" s="5"/>
+      <x:c r="C111" s="3" t="str">
+        <x:v>Q4 revenue needed (USD bn)</x:v>
+      </x:c>
+      <x:c r="D111" s="125" t="n">
+        <x:f>D110-D109</x:f>
+        <x:v>30.9</x:v>
+      </x:c>
       <x:c r="E111" s="5"/>
       <x:c r="F111" s="5"/>
       <x:c r="G111" s="5"/>
@@ -3905,8 +3937,13 @@
     <x:row r="112" ht="21" customHeight="1">
       <x:c r="A112" s="3"/>
       <x:c r="B112" s="3"/>
-      <x:c r="C112" s="3"/>
-      <x:c r="D112" s="5"/>
+      <x:c r="C112" s="3" t="str">
+        <x:v>Required Q4 growth vs Q3</x:v>
+      </x:c>
+      <x:c r="D112" s="126" t="n">
+        <x:f>D111/'Inputs'!J39-1</x:f>
+        <x:v>0.8392857142857142</x:v>
+      </x:c>
       <x:c r="E112" s="5"/>
       <x:c r="F112" s="5"/>
       <x:c r="G112" s="5"/>
@@ -4220,7 +4257,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8efd57df475471d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40d1579a417e4415"/>
 </x:worksheet>
 </file>
 
@@ -7211,11 +7248,11 @@
         <x:v>Research cutoff</x:v>
       </x:c>
       <x:c r="D8" s="17" t="d">
-        <x:v>2026-10-11T00:00:00.000Z</x:v>
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E8" s="4"/>
       <x:c r="F8" s="26" t="str">
-        <x:v>Public S-1 had not posted to EDGAR as of 9 Oct 2026 [S8]. No audited financials exist yet.</x:v>
+        <x:v>Reviewed through 16 Oct 2026 Beijing time; latest observations in S18/S19.</x:v>
       </x:c>
       <x:c r="G8" s="4"/>
       <x:c r="H8" s="4"/>
@@ -7367,11 +7404,11 @@
       </x:c>
       <x:c r="D15" s="18" t="n">
         <x:f>D45</x:f>
-        <x:v>2000</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="E15" s="4"/>
       <x:c r="F15" s="26" t="str">
-        <x:v>$2tn reference from September reporting [S3]. Not a priced offer.</x:v>
+        <x:v>Investor discussion reported 16 Oct Beijing time [S18]; not a priced offer.</x:v>
       </x:c>
       <x:c r="G15" s="4"/>
       <x:c r="H15" s="4"/>
@@ -7751,7 +7788,7 @@
       <x:c r="A29" s="3"/>
       <x:c r="B29" s="3"/>
       <x:c r="C29" s="40" t="str">
-        <x:v>2026 revenue of $64bn is a model output, not a disclosure. It integrates the published run-rate path</x:v>
+        <x:v>2026 revenue of USD64bn remains an analyst assumption, not a reported annual result.</x:v>
       </x:c>
       <x:c r="D29" s="5"/>
       <x:c r="E29" s="5"/>
@@ -7769,7 +7806,7 @@
       <x:c r="A30" s="3"/>
       <x:c r="B30" s="3"/>
       <x:c r="C30" s="40" t="str">
-        <x:v>($9bn Dec-25, $20bn Mar-26, $30bn Apr-26, $47bn May-26, $65bn Jul-26, $100-120bn Dec-26E) over twelve months.</x:v>
+        <x:v>Latest quarterly observations and a full-year reconciliation appear below and on Valuation.</x:v>
       </x:c>
       <x:c r="D30" s="5"/>
       <x:c r="E30" s="5"/>
@@ -7890,11 +7927,21 @@
         <x:v>Source ID</x:v>
       </x:c>
       <x:c r="H36" s="5"/>
-      <x:c r="I36" s="5"/>
-      <x:c r="J36" s="5"/>
-      <x:c r="K36" s="5"/>
-      <x:c r="L36" s="5"/>
-      <x:c r="M36" s="5"/>
+      <x:c r="I36" s="32" t="str">
+        <x:v>Period</x:v>
+      </x:c>
+      <x:c r="J36" s="43" t="str">
+        <x:v>Revenue $bn</x:v>
+      </x:c>
+      <x:c r="K36" s="43" t="str">
+        <x:v>Available BJT</x:v>
+      </x:c>
+      <x:c r="L36" s="43" t="str">
+        <x:v>Classification</x:v>
+      </x:c>
+      <x:c r="M36" s="43" t="str">
+        <x:v>Source</x:v>
+      </x:c>
       <x:c r="N36" s="5"/>
     </x:row>
     <x:row r="37" ht="21" customHeight="1">
@@ -7916,11 +7963,21 @@
         <x:v>S3</x:v>
       </x:c>
       <x:c r="H37" s="5"/>
-      <x:c r="I37" s="5"/>
-      <x:c r="J37" s="5"/>
-      <x:c r="K37" s="5"/>
-      <x:c r="L37" s="5"/>
-      <x:c r="M37" s="5"/>
+      <x:c r="I37" s="3" t="str">
+        <x:v>2026Q1</x:v>
+      </x:c>
+      <x:c r="J37" s="123" t="n">
+        <x:v>4.7</x:v>
+      </x:c>
+      <x:c r="K37" s="124" t="d">
+        <x:v>2026-10-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L37" s="4" t="str">
+        <x:v>Media-reported</x:v>
+      </x:c>
+      <x:c r="M37" s="4" t="str">
+        <x:v>S19</x:v>
+      </x:c>
       <x:c r="N37" s="5"/>
     </x:row>
     <x:row r="38" ht="21" customHeight="1">
@@ -7942,11 +7999,21 @@
         <x:v>S3</x:v>
       </x:c>
       <x:c r="H38" s="5"/>
-      <x:c r="I38" s="5"/>
-      <x:c r="J38" s="5"/>
-      <x:c r="K38" s="5"/>
-      <x:c r="L38" s="5"/>
-      <x:c r="M38" s="5"/>
+      <x:c r="I38" s="3" t="str">
+        <x:v>2026Q2</x:v>
+      </x:c>
+      <x:c r="J38" s="123" t="n">
+        <x:v>11.6</x:v>
+      </x:c>
+      <x:c r="K38" s="124" t="d">
+        <x:v>2026-10-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L38" s="4" t="str">
+        <x:v>Media-reported</x:v>
+      </x:c>
+      <x:c r="M38" s="4" t="str">
+        <x:v>S19</x:v>
+      </x:c>
       <x:c r="N38" s="5"/>
     </x:row>
     <x:row r="39" ht="21" customHeight="1">
@@ -7968,11 +8035,21 @@
         <x:v>S1</x:v>
       </x:c>
       <x:c r="H39" s="5"/>
-      <x:c r="I39" s="5"/>
-      <x:c r="J39" s="5"/>
-      <x:c r="K39" s="5"/>
-      <x:c r="L39" s="5"/>
-      <x:c r="M39" s="5"/>
+      <x:c r="I39" s="3" t="str">
+        <x:v>2026Q3</x:v>
+      </x:c>
+      <x:c r="J39" s="123" t="n">
+        <x:v>16.8</x:v>
+      </x:c>
+      <x:c r="K39" s="124" t="d">
+        <x:v>2026-10-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L39" s="4" t="str">
+        <x:v>Media-reported</x:v>
+      </x:c>
+      <x:c r="M39" s="4" t="str">
+        <x:v>S19</x:v>
+      </x:c>
       <x:c r="N39" s="5"/>
     </x:row>
     <x:row r="40" ht="21" customHeight="1">
@@ -8109,19 +8186,19 @@
       <x:c r="A45" s="3"/>
       <x:c r="B45" s="3"/>
       <x:c r="C45" s="3" t="str">
-        <x:v>IPO equity benchmark, about</x:v>
+        <x:v>IPO investor discussion, about</x:v>
       </x:c>
       <x:c r="D45" s="44" t="n">
-        <x:v>2000</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="E45" s="45" t="str">
-        <x:v>Sep-26</x:v>
+        <x:v>16-Oct-26 BJT</x:v>
       </x:c>
       <x:c r="F45" s="4" t="str">
-        <x:v>Reported target</x:v>
+        <x:v>Media-reported</x:v>
       </x:c>
       <x:c r="G45" s="4" t="str">
-        <x:v>S3</x:v>
+        <x:v>S18</x:v>
       </x:c>
       <x:c r="H45" s="5"/>
       <x:c r="I45" s="5"/>
@@ -8135,19 +8212,19 @@
       <x:c r="A46" s="3"/>
       <x:c r="B46" s="3"/>
       <x:c r="C46" s="3" t="str">
-        <x:v>Long-term compute commitments, over</x:v>
+        <x:v>Long-term compute commitments, at least</x:v>
       </x:c>
       <x:c r="D46" s="44" t="n">
-        <x:v>417</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="E46" s="45" t="str">
-        <x:v>Early 2026</x:v>
+        <x:v>Oct-26</x:v>
       </x:c>
       <x:c r="F46" s="4" t="str">
         <x:v>Media-reported</x:v>
       </x:c>
       <x:c r="G46" s="4" t="str">
-        <x:v>S3</x:v>
+        <x:v>S19</x:v>
       </x:c>
       <x:c r="H46" s="5"/>
       <x:c r="I46" s="5"/>
@@ -9664,7 +9741,9 @@
     <x:row r="125" ht="21" customHeight="1">
       <x:c r="A125" s="3"/>
       <x:c r="B125" s="3"/>
-      <x:c r="C125" s="3"/>
+      <x:c r="C125" s="3" t="str">
+        <x:v>S18. Reuters, 15 Oct 21:00 UTC / 16 Oct 05:00 Beijing. IPO investor discussion.</x:v>
+      </x:c>
       <x:c r="D125" s="5"/>
       <x:c r="E125" s="5"/>
       <x:c r="F125" s="5"/>
@@ -9680,7 +9759,9 @@
     <x:row r="126" ht="21" customHeight="1">
       <x:c r="A126" s="3"/>
       <x:c r="B126" s="3"/>
-      <x:c r="C126" s="3"/>
+      <x:c r="C126" s="3" t="str">
+        <x:v>https://www.aol.com/articles/exclusive-investors-temper-anthropic-ipo-210007000.html</x:v>
+      </x:c>
       <x:c r="D126" s="5"/>
       <x:c r="E126" s="5"/>
       <x:c r="F126" s="5"/>
@@ -9712,7 +9793,9 @@
     <x:row r="128" ht="21" customHeight="1">
       <x:c r="A128" s="3"/>
       <x:c r="B128" s="3"/>
-      <x:c r="C128" s="3"/>
+      <x:c r="C128" s="3" t="str">
+        <x:v>S19. Reuters, 15 Oct Beijing. Quarterly revenue and decade-long compute commitments.</x:v>
+      </x:c>
       <x:c r="D128" s="5"/>
       <x:c r="E128" s="5"/>
       <x:c r="F128" s="5"/>
@@ -9728,7 +9811,9 @@
     <x:row r="129" ht="21" customHeight="1">
       <x:c r="A129" s="3"/>
       <x:c r="B129" s="3"/>
-      <x:c r="C129" s="3"/>
+      <x:c r="C129" s="3" t="str">
+        <x:v>https://uk.marketscreener.com/news/anthropic-s-q3-revenue-surges-45-to-nearly-17-billion-ce785dd2d08cf221</x:v>
+      </x:c>
       <x:c r="D129" s="5"/>
       <x:c r="E129" s="5"/>
       <x:c r="F129" s="5"/>

</xml_diff>